<commit_message>
Atualiza universo Spot v2.1
Atualiza universo Spot v2.1 e restaura timeframes configuráveis
</commit_message>
<xml_diff>
--- a/ativos_spot.xlsx
+++ b/ativos_spot.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ATIVOS" sheetId="1" r:id="R3ce5bc9eab614b09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SPOT" sheetId="2" r:id="Rc510c9d16a8847e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FILTROS_SPOT" sheetId="3" r:id="Rd06e656ddfd949db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ATIVOS" sheetId="1" r:id="R726fa3f268194c0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_UNIVERSO" sheetId="2" r:id="R6baf94470c224b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SPOT" sheetId="3" r:id="Rc5da5214305c431e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FILTROS_SPOT" sheetId="4" r:id="Rf787391fa1db40b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36,7 +37,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1F4E78"/>
+        <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -47,7 +48,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -69,10 +70,22 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -295,21 +308,21 @@
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="7" t="str">
         <x:v>ATIVO</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="7" t="str">
         <x:v>Par</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="7" t="str">
         <x:v>Timeframe</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="7" t="str">
         <x:v>Mercado</x:v>
       </x:c>
     </x:row>
@@ -384,38 +397,140 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="A2:A1000">
-      <x:formula1>"true,false"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="C2:C1000">
-      <x:formula1>"120,240,D"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="D2:D1000">
-      <x:formula1>"spot"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="68" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="7" t="str">
+        <x:v>Parâmetro</x:v>
+      </x:c>
+      <x:c r="B1" s="7" t="str">
+        <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="C1" s="7" t="str">
+        <x:v>Observação</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>MODO_UNIVERSO</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>HIBRIDO</x:v>
+      </x:c>
+      <x:c r="C2" s="12" t="str">
+        <x:v>AUTO | HIBRIDO | MANUAL. Pode ser sobrescrito pela linha de comando.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>TIMEFRAMES_PADRAO</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>120,240,360,D</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="str">
+        <x:v>Aplicados a cada ativo elegível em AUTO/HIBRIDO. Intervalos Bybit V5 válidos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>HISTORICO_MIN_DIAS</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="str">
+        <x:v>Substitui IDADE_MIN_DIAS no Spot. Exige evidência de negociação há pelo menos este número de dias.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>KLINE_LIMIT</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
+        <x:v>Quantidade de candles baixados por par/timeframe no scan técnico (máx. 1000 por chamada).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>EXCLUIR_STABLECOINS</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>SIM</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
+        <x:v>Exclui pares cuja moeda-base esteja na lista STABLECOINS_EXCLUIR.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>STABLECOINS_EXCLUIR</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>USDT,USDC,DAI,FDUSD,TUSD,PYUSD,USDE,USD1,USDS,EURC</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
+        <x:v>Lista editável de moedas-base a excluir.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>EXCLUIR_ST_TAG</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>SIM</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
+        <x:v>Exclui instrumentos Spot com stTag=1 (Special Treatment).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>SYMBOL_TYPES_EXCLUIR</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>xstocks</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>Tipos Spot a excluir. Deixe vazio para não filtrar por symbolType.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="7" t="str">
         <x:v>Parâmetro</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="7" t="str">
         <x:v>Valor inicial</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="7" t="str">
         <x:v>Observação</x:v>
       </x:c>
     </x:row>
@@ -426,7 +541,7 @@
       <x:c r="B2" t="str">
         <x:v>spot</x:v>
       </x:c>
-      <x:c r="C2" t="str">
+      <x:c r="C2" s="12" t="str">
         <x:v>Fixo</x:v>
       </x:c>
     </x:row>
@@ -437,7 +552,7 @@
       <x:c r="B3" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="C3" t="str">
+      <x:c r="C3" s="12" t="str">
         <x:v>Taxa por lado; ajuste ao seu nível na Bybit</x:v>
       </x:c>
     </x:row>
@@ -448,7 +563,7 @@
       <x:c r="B4" t="n">
         <x:v>0.15</x:v>
       </x:c>
-      <x:c r="C4" t="str">
+      <x:c r="C4" s="12" t="str">
         <x:v>Lucro líquido mínimo estimado por ciclo de grid</x:v>
       </x:c>
     </x:row>
@@ -459,7 +574,7 @@
       <x:c r="B5" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C5" t="str">
+      <x:c r="C5" s="12" t="str">
         <x:v>ATR usado na parametrização</x:v>
       </x:c>
     </x:row>
@@ -470,7 +585,7 @@
       <x:c r="B6" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C6" t="str">
+      <x:c r="C6" s="12" t="str">
         <x:v>Limite inferior = entry - fator × ATR</x:v>
       </x:c>
     </x:row>
@@ -481,7 +596,7 @@
       <x:c r="B7" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C7" t="str">
+      <x:c r="C7" s="12" t="str">
         <x:v>Limite superior = entry + fator × ATR</x:v>
       </x:c>
     </x:row>
@@ -492,7 +607,7 @@
       <x:c r="B8" t="n">
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="C8" t="str">
+      <x:c r="C8" s="12" t="str">
         <x:v>SL fica abaixo do limite inferior</x:v>
       </x:c>
     </x:row>
@@ -503,7 +618,7 @@
       <x:c r="B9" t="n">
         <x:v>0.7</x:v>
       </x:c>
-      <x:c r="C9" t="str">
+      <x:c r="C9" s="12" t="str">
         <x:v>TP fica acima do limite superior</x:v>
       </x:c>
     </x:row>
@@ -514,7 +629,7 @@
       <x:c r="B10" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C10" t="str">
+      <x:c r="C10" s="12" t="str">
         <x:v>Piso operacional</x:v>
       </x:c>
     </x:row>
@@ -525,30 +640,8 @@
       <x:c r="B11" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="C11" t="str">
+      <x:c r="C11" s="12" t="str">
         <x:v>Teto de recomendação</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>SLOPE_TRAILING_UP</x:v>
-      </x:c>
-      <x:c r="B12" t="n">
-        <x:v>0.75</x:v>
-      </x:c>
-      <x:c r="C12" t="str">
-        <x:v>Acima disso sugere Trailing Up</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>VENDA</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>AGUARDAR/SAIR</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
-        <x:v>Nunca converter em SHORT no Spot</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -556,27 +649,27 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="9.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="8.5" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="5" t="str">
+      <x:c r="A1" s="7" t="str">
         <x:v>Filtro</x:v>
       </x:c>
-      <x:c r="B1" s="5" t="str">
+      <x:c r="B1" s="7" t="str">
         <x:v>Valor inicial</x:v>
       </x:c>
-      <x:c r="C1" s="5" t="str">
+      <x:c r="C1" s="7" t="str">
         <x:v>Prioridade</x:v>
       </x:c>
-      <x:c r="D1" s="5" t="str">
+      <x:c r="D1" s="7" t="str">
         <x:v>Comentário</x:v>
       </x:c>
     </x:row>
@@ -590,7 +683,7 @@
       <x:c r="C2" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D2" t="str">
+      <x:c r="D2" s="12" t="str">
         <x:v>Mantido; agora exclusivamente Spot</x:v>
       </x:c>
     </x:row>
@@ -604,7 +697,7 @@
       <x:c r="C3" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D3" t="str">
+      <x:c r="D3" s="12" t="str">
         <x:v>Mantido; book Spot</x:v>
       </x:c>
     </x:row>
@@ -618,7 +711,7 @@
       <x:c r="C4" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D4" t="str">
+      <x:c r="D4" s="12" t="str">
         <x:v>Mantido; book Spot</x:v>
       </x:c>
     </x:row>
@@ -632,7 +725,7 @@
       <x:c r="C5" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D5" t="str">
+      <x:c r="D5" s="12" t="str">
         <x:v>Recalibrar após primeira amostra Spot</x:v>
       </x:c>
     </x:row>
@@ -646,7 +739,7 @@
       <x:c r="C6" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D6" t="str">
+      <x:c r="D6" s="12" t="str">
         <x:v>Evita volatilidade excessiva</x:v>
       </x:c>
     </x:row>
@@ -660,7 +753,7 @@
       <x:c r="C7" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D7" t="str">
+      <x:c r="D7" s="12" t="str">
         <x:v>Classifica alta/Trailing Up</x:v>
       </x:c>
     </x:row>
@@ -674,7 +767,7 @@
       <x:c r="C8" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D8" t="str">
+      <x:c r="D8" s="12" t="str">
         <x:v>Não se aplica a Spot</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Ajuste Filtro de ativos_spot.xlsx
</commit_message>
<xml_diff>
--- a/ativos_spot.xlsx
+++ b/ativos_spot.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\INVESTIMENTOS VARIAVEL\Bybit\bybit_setups\complementos\GitHub\bybit_setups\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\INVESTIMENTOS VARIAVEL\Bybit\bybit_setups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45041EA6-E626-4713-A6D2-4B8DA762C684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C4D906-5F2D-4EA2-8933-25A4FC426167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6360" yWindow="1392" windowWidth="11448" windowHeight="8964" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10932" yWindow="1296" windowWidth="11448" windowHeight="8964" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ATIVOS" sheetId="1" r:id="rId1"/>
@@ -952,7 +952,7 @@
         <v>65</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="C5">
         <v>2</v>

</xml_diff>